<commit_message>
Update public download template with the cleaner Excel file
</commit_message>
<xml_diff>
--- a/public/BPCL_Welcome_Poster_Template.xlsx
+++ b/public/BPCL_Welcome_Poster_Template.xlsx
@@ -5,69 +5,38 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/apple/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9302007939da05d8/The Strategist/Personal/Antigravity/BPCL - Poster/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D8ED8A7F-8F9A-0D40-A820-10C6A8237870}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{234D2738-E08D-B649-8DB3-14073593FC42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
-  <metadataTypes count="1">
-    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLRICHVALUE" count="3">
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="0"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="1"/>
-        </ext>
-      </extLst>
-    </bk>
-    <bk>
-      <extLst>
-        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
-          <xlrd:rvb i="2"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <valueMetadata count="3">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-    <bk>
-      <rc t="1" v="1"/>
-    </bk>
-    <bk>
-      <rc t="1" v="2"/>
-    </bk>
-  </valueMetadata>
-</metadata>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>Email</t>
   </si>
@@ -93,80 +62,13 @@
     <t>Mobile No.</t>
   </si>
   <si>
-    <t>Athul K N</t>
-  </si>
-  <si>
-    <t>24255</t>
-  </si>
-  <si>
-    <t>9+ Years</t>
-  </si>
-  <si>
-    <t>Senior Reliability Engineer at Dow Chemicals International Chennai</t>
-  </si>
-  <si>
-    <t>Father, Mother and one younger brother</t>
-  </si>
-  <si>
-    <t>Travelling, Fishing, Cricket, Movies, Music</t>
-  </si>
-  <si>
-    <t>8281023128</t>
-  </si>
-  <si>
-    <t>Harikrishnan Pu</t>
-  </si>
-  <si>
-    <t>24256</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8 YEARS </t>
-  </si>
-  <si>
-    <t>SENIOR ELECTRICAL ENGINEER AT HOCL,AMBALAMUGAL</t>
-  </si>
-  <si>
-    <t>WIFE:DILNA A,MOTHER:SHANI UNNI, FATHER:UNNI PK,BROTHER:SHYAM MOHAN</t>
-  </si>
-  <si>
-    <t>PHOTOGRAPHY AND TRAVELLING</t>
-  </si>
-  <si>
-    <t>8593953836</t>
-  </si>
-  <si>
-    <t>Potnuru Shyam Shankar</t>
-  </si>
-  <si>
-    <t>24466</t>
-  </si>
-  <si>
-    <t>1. Good Experience in production department - Roles - Field Coordinator, Panel Operator for urea plant &amp; Shiftincharge for Urea, Nitric Acid, Ammonium Nitrate plants.
-2. Good Experience in Project, Precommissioning and little commissioning activities for Nitric Acid/Technical Ammonium Nitrate Project.</t>
-  </si>
-  <si>
-    <t>Assistant Manager at Chambal Fertilizers and Chemicals Limited</t>
-  </si>
-  <si>
-    <t>Mother - Potnuru Parvathi(Housewife), Father - Potnuru Anand(Expired), Sister - Chinnari Anusha(Married)married</t>
-  </si>
-  <si>
-    <t>Watching Movies/Webseries, Cooking Food, Playing Cricket, Carroms.</t>
-  </si>
-  <si>
-    <t>7981159057</t>
-  </si>
-  <si>
     <t>Designation</t>
   </si>
   <si>
     <t>Date of Joining</t>
   </si>
   <si>
-    <t>ASSOCIATE EXECUTIVE (ENGINEERING)</t>
-  </si>
-  <si>
-    <t>ajaythomas@gmail.com</t>
+    <t>Photo</t>
   </si>
 </sst>
 </file>
@@ -270,7 +172,10 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="9">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -308,94 +213,21 @@
 </styleSheet>
 </file>
 
-<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
-<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
-  <global>
-    <keyFlags>
-      <key name="_Self">
-        <flag name="ExcludeFromFile" value="1"/>
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_DisplayString">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Flags">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Format">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_SubLabel">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Attribution">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Icon">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_Display">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_CanonicalPropertyNames">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-      <key name="_ClassificationId">
-        <flag name="ExcludeFromCalcComparison" value="1"/>
-      </key>
-    </keyFlags>
-  </global>
-</rvTypesInfo>
-</file>
-
-<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
-<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="3">
-  <rv s="0">
-    <v>0</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>1</v>
-    <v>5</v>
-  </rv>
-  <rv s="0">
-    <v>2</v>
-    <v>5</v>
-  </rv>
-</rvData>
-</file>
-
-<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
-<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
-  <s t="_localImage">
-    <k n="_rvRel:LocalImageIdentifier" t="i"/>
-    <k n="CalcOrigin" t="i"/>
-  </s>
-</rvStructures>
-</file>
-
-<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
-<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <rel r:id="rId1"/>
-  <rel r:id="rId2"/>
-  <rel r:id="rId3"/>
-</richValueRels>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:J4" totalsRowShown="0">
-  <autoFilter ref="A1:J4" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="10">
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Staff No." dataDxfId="5"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:K2" insertRow="1" totalsRowShown="0">
+  <autoFilter ref="A1:K2" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="11">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Name" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Staff No." dataDxfId="6"/>
     <tableColumn id="3" xr3:uid="{94496847-35BC-442F-A1A1-FACBC6820CF4}" name="Designation"/>
     <tableColumn id="2" xr3:uid="{B9D784D0-26C6-4233-B75F-4B349E285456}" name="Date of Joining"/>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Experience" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Previous Job" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Details of Family Members" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Hobbies &amp; Interest " dataDxfId="1"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Mobile No." dataDxfId="0"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Experience" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Previous Job" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Details of Family Members" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Hobbies &amp; Interest " dataDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Mobile No." dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{E674DE21-8C68-7246-992A-225AE28CDF3A}" name="Photo" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -698,7 +530,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45.5" bestFit="1" customWidth="1"/>
@@ -723,10 +555,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
@@ -743,122 +575,22 @@
       <c r="J1" t="s">
         <v>7</v>
       </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" ht="26" x14ac:dyDescent="0.2">
-      <c r="A2" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="5">
-        <v>46140</v>
-      </c>
-      <c r="F2" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" t="s">
-        <v>12</v>
-      </c>
-      <c r="I2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="K2" t="e" vm="1">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" ht="26" x14ac:dyDescent="0.2">
-      <c r="A3" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E3" s="5">
-        <v>46137</v>
-      </c>
-      <c r="F3" t="s">
-        <v>17</v>
-      </c>
-      <c r="G3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" t="s">
-        <v>20</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="K3" t="e" vm="2">
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="26" x14ac:dyDescent="0.2">
-      <c r="A4" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="B4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" s="5">
-        <v>46167</v>
-      </c>
-      <c r="F4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G4" t="s">
-        <v>25</v>
-      </c>
-      <c r="H4" t="s">
-        <v>26</v>
-      </c>
-      <c r="I4" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="K4" t="e" vm="3">
-        <v>#VALUE!</v>
-      </c>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A2" s="6"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="5"/>
+      <c r="J2" s="1"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{645C5DA2-8A80-B845-A432-3B84AB52827B}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{63CF30EC-4C29-0E4F-B238-2CC4900544B3}"/>
-    <hyperlink ref="A4" r:id="rId3" xr:uid="{1ED73588-5E24-2441-98CB-12C4E88C1B55}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>